<commit_message>
first set of conclusions
</commit_message>
<xml_diff>
--- a/data/metadata.xlsx
+++ b/data/metadata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://o365coloradoedu-my.sharepoint.com/personal/stta6032_colorado_edu/Documents/Documents/GitHub/Lake-Trout-AK/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="8_{CCB36ED4-EE71-4D46-BB62-C8EE1AA7C738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F60EBE3-BEFC-4236-ACF7-392D26D76D77}"/>
+  <xr:revisionPtr revIDLastSave="55" documentId="8_{CCB36ED4-EE71-4D46-BB62-C8EE1AA7C738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F0D23F43-7D3C-40CE-9F54-B97B27B9D9F0}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{E28188F2-719D-475E-9847-354F5D067B84}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
   <si>
     <t>Run</t>
   </si>
@@ -44,43 +44,100 @@
     <t>Run_name</t>
   </si>
   <si>
-    <t>Age 10</t>
-  </si>
-  <si>
-    <t>Age 12</t>
-  </si>
-  <si>
-    <t>Age 13</t>
-  </si>
-  <si>
-    <t>Age 14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Age 15 </t>
-  </si>
-  <si>
-    <t>Age 16</t>
-  </si>
-  <si>
-    <t>Age 18</t>
-  </si>
-  <si>
-    <t>Age 19</t>
-  </si>
-  <si>
-    <t>Age 20</t>
-  </si>
-  <si>
-    <t>Age 23</t>
-  </si>
-  <si>
-    <t>Age 24</t>
-  </si>
-  <si>
-    <t>Age 26</t>
-  </si>
-  <si>
-    <t>Age 56</t>
+    <t>Age 12 mean</t>
+  </si>
+  <si>
+    <t>Age 12 lower 1 SD</t>
+  </si>
+  <si>
+    <t>Age 12 lower 2 SD</t>
+  </si>
+  <si>
+    <t>Age 12 upper 1 SD</t>
+  </si>
+  <si>
+    <t>Age 12 upper 2 SD</t>
+  </si>
+  <si>
+    <t>Age 12 upper 3 SD</t>
+  </si>
+  <si>
+    <t>Age 13 mean</t>
+  </si>
+  <si>
+    <t>Age 13 lower 1 SD</t>
+  </si>
+  <si>
+    <t>Age 13 lower 2 SD</t>
+  </si>
+  <si>
+    <t>Age 13 upper 1 SD</t>
+  </si>
+  <si>
+    <t>Age 13 upper 2 SD</t>
+  </si>
+  <si>
+    <t>Age 13 upper 3 SD</t>
+  </si>
+  <si>
+    <t>Age 14 mean</t>
+  </si>
+  <si>
+    <t>Age 14 lower 1 SD</t>
+  </si>
+  <si>
+    <t>Age 14 lower 2 SD</t>
+  </si>
+  <si>
+    <t>Age 14 lower 3 SD</t>
+  </si>
+  <si>
+    <t>Age 14 upper 1 SD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Age 14 upper 2 SD </t>
+  </si>
+  <si>
+    <t>Age 14 upper 3 SD</t>
+  </si>
+  <si>
+    <t>Age 18 mean</t>
+  </si>
+  <si>
+    <t>Age 18 lower 1 SD</t>
+  </si>
+  <si>
+    <t>Age 18 lower 2 SD</t>
+  </si>
+  <si>
+    <t>Age 18 lower 3 SD</t>
+  </si>
+  <si>
+    <t>Age 18 upper 1 SD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Age 18 upper 2 SD </t>
+  </si>
+  <si>
+    <t>Age 18 upper 3 SD</t>
+  </si>
+  <si>
+    <t>Age 23 mean</t>
+  </si>
+  <si>
+    <t>Age 23 lower 1 SD</t>
+  </si>
+  <si>
+    <t>Age 23 lower 2 SD</t>
+  </si>
+  <si>
+    <t>Age 23 upper 1 SD</t>
+  </si>
+  <si>
+    <t>Age 23 upper 2 SD</t>
+  </si>
+  <si>
+    <t>Age 23 upper 3 SD</t>
   </si>
 </sst>
 </file>
@@ -452,7 +509,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16C8752E-AA33-4EF2-B526-239F3383BACD}">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -567,6 +624,158 @@
         <v>14</v>
       </c>
     </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>